<commit_message>
Refresh publications data from OpenAlex
Automated weekly refresh.
</commit_message>
<xml_diff>
--- a/papers.xlsx
+++ b/papers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -467,16 +467,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Accessible, Realistic Genome Simulation with Selection Using stdpopsim</t>
+          <t>Efficient ancestry and mutation simulation with msprime 1.0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Molecular Biology and Evolution</t>
+          <t>UNC Libraries</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -485,11 +485,11 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Graham Gower, Nathaniel S. Pope, Murillo F. Rodrigues, Silas Tittes, Linh N Tran, Ornob Alam, Maria Izabel A. Cavassim, Peter D. Fields</t>
+          <t>Jared Galloway, Bjarki Eldon, Ariella Gladstein, Daniel Goldstein, Andrew D. Kern, Yan Wong, Nathaniel S. Pope, Consuelo D. Quinto-Cortés</t>
         </is>
       </c>
     </row>
@@ -498,16 +498,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>link-ancestors: fast simulation of local ancestry with tree sequence software</t>
+          <t>Accessible, Realistic Genome Simulation with Selection Using stdpopsim</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bioinformatics Advances</t>
+          <t>Molecular Biology and Evolution</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -516,11 +516,11 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Jerome Kelleher, Peter L. Ralph, Stephen Leslie, Damjan Vukcevic</t>
+          <t>Graham Gower, Nathaniel S. Pope, Murillo F. Rodrigues, Silas Tittes, Linh N Tran, Ornob Alam, Maria Izabel A. Cavassim, Peter D. Fields</t>
         </is>
       </c>
     </row>
@@ -533,12 +533,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Indigenous Australian genomes show deep structure and rich novel variation</t>
+          <t>link-ancestors: fast simulation of local ancestry with tree sequence software</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Bioinformatics Advances</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -547,11 +547,11 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>77</v>
+        <v>15</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Matthew Silcocks, Ashley Farlow, Azure Hermes, Hardip R. Patel, Sharon Huebner, Gareth Baynam, Misty R. Jenkins, Damjan Vukcevic</t>
+          <t>Jerome Kelleher, Peter L. Ralph, Stephen Leslie, Damjan Vukcevic</t>
         </is>
       </c>
     </row>
@@ -564,12 +564,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Expanding the stdpopsim species catalog, and lessons learned for realistic genome simulations</t>
+          <t>Indigenous Australian genomes show deep structure and rich novel variation</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>eLife</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -578,11 +578,11 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>M. Elise Lauterbur, Maria Izabel A. Cavassim, Ariella Gladstein, Graham Gower, Nathaniel S. Pope, Jeffrey R. Adrion, Saurabh Belsare, Arjun Biddanda</t>
+          <t>Matthew Silcocks, Ashley Farlow, Azure Hermes, Hardip R. Patel, Sharon Huebner, Gareth Baynam, Misty R. Jenkins, Damjan Vukcevic</t>
         </is>
       </c>
     </row>
@@ -591,16 +591,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Efficient ancestry and mutation simulation with msprime 1.0</t>
+          <t>Expanding the stdpopsim species catalog, and lessons learned for realistic genome simulations</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Genetics</t>
+          <t>eLife</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -609,11 +609,11 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>539</v>
+        <v>55</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Franz Baumdicker, Gertjan Bisschop, Daniel Goldstein, Graham Gower, Aaron P. Ragsdale, Sha Zhu, Bjarki Eldon, E. Castedo Ellerman</t>
+          <t>M. Elise Lauterbur, Maria Izabel A. Cavassim, Ariella Gladstein, Graham Gower, Nathaniel S. Pope, Jeffrey R. Adrion, Saurabh Belsare, Arjun Biddanda</t>
         </is>
       </c>
     </row>
@@ -622,27 +622,58 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Efficient ancestry and mutation simulation with msprime 1.0</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Genetics</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>539</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Franz Baumdicker, Gertjan Bisschop, Daniel Goldstein, Graham Gower, Aaron P. Ragsdale, Sha Zhu, Bjarki Eldon, E. Castedo Ellerman</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
         <v>2020</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>A community-maintained standard library of population genetic models</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>eLife</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>article</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F8" t="n">
         <v>268</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Jeffrey R. Adrion, C. B. Cole, Noah Dukler, Jared Galloway, Ariella Gladstein, Graham Gower, Christopher C. Kyriazis, Aaron P. Ragsdale</t>
         </is>

</xml_diff>